<commit_message>
just reran the model
</commit_message>
<xml_diff>
--- a/household_income_model_comparison.xlsx
+++ b/household_income_model_comparison.xlsx
@@ -11,71 +11,6 @@
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
-  <si>
-    <t>model</t>
-  </si>
-  <si>
-    <t>k</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
-    <t>param2</t>
-  </si>
-  <si>
-    <t>param2_name</t>
-  </si>
-  <si>
-    <t>lambda</t>
-  </si>
-  <si>
-    <t>epsilon</t>
-  </si>
-  <si>
-    <t>logLik</t>
-  </si>
-  <si>
-    <t>AIC</t>
-  </si>
-  <si>
-    <t>BIC</t>
-  </si>
-  <si>
-    <t>n_converged</t>
-  </si>
-  <si>
-    <t>n_tries</t>
-  </si>
-  <si>
-    <t>convergence_rate</t>
-  </si>
-  <si>
-    <t>AIC_rank</t>
-  </si>
-  <si>
-    <t>BIC_rank</t>
-  </si>
-  <si>
-    <t>cmLN</t>
-  </si>
-  <si>
-    <t>sigma</t>
-  </si>
-  <si>
-    <t>mG</t>
-  </si>
-  <si>
-    <t>shape</t>
-  </si>
-  <si>
-    <t>mIG</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -416,59 +351,91 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>param2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>param2_name</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>lambda</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>epsilon</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>logLik</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>AIC</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>BIC</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>n_converged</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>n_tries</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>convergence_rate</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>AIC_rank</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>BIC_rank</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:15">
-      <c r="A2" t="s">
-        <v>15</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>cmLN</t>
+        </is>
       </c>
       <c r="B2">
         <v>4</v>
@@ -479,8 +446,10 @@
       <c r="D2">
         <v>0.8250999999999999</v>
       </c>
-      <c r="E2" t="s">
-        <v>16</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>sigma</t>
+        </is>
       </c>
       <c r="F2">
         <v>1.9445</v>
@@ -513,30 +482,34 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
-      <c r="A3" t="s">
-        <v>17</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>mLN</t>
+        </is>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3">
-        <v>0.038</v>
+        <v>29593.3686</v>
       </c>
       <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>18</v>
+        <v>1.0555</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>sigma</t>
+        </is>
       </c>
       <c r="H3">
-        <v>-259357.4168</v>
+        <v>-256879.0957</v>
       </c>
       <c r="I3">
-        <v>518718.8336</v>
+        <v>513762.1914</v>
       </c>
       <c r="J3">
-        <v>518734.6346</v>
+        <v>513777.9924</v>
       </c>
       <c r="K3">
         <v>50</v>
@@ -548,36 +521,40 @@
         <v>1</v>
       </c>
       <c r="N3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
-      <c r="A4" t="s">
-        <v>19</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mG</t>
+        </is>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4">
-        <v>22077.6427</v>
+        <v>0.038</v>
       </c>
       <c r="D4">
-        <v>67457.72900000001</v>
-      </c>
-      <c r="E4" t="s">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>shape</t>
+        </is>
       </c>
       <c r="H4">
-        <v>-258694.6226</v>
+        <v>-259357.4168</v>
       </c>
       <c r="I4">
-        <v>517393.2453</v>
+        <v>518718.8336</v>
       </c>
       <c r="J4">
-        <v>517409.0462</v>
+        <v>518734.6346</v>
       </c>
       <c r="K4">
         <v>50</v>
@@ -589,10 +566,55 @@
         <v>1</v>
       </c>
       <c r="N4">
+        <v>4</v>
+      </c>
+      <c r="O4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mIG</t>
+        </is>
+      </c>
+      <c r="B5">
         <v>2</v>
       </c>
-      <c r="O4">
-        <v>2</v>
+      <c r="C5">
+        <v>22077.6427</v>
+      </c>
+      <c r="D5">
+        <v>67457.72900000001</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>lambda</t>
+        </is>
+      </c>
+      <c r="H5">
+        <v>-258694.6226</v>
+      </c>
+      <c r="I5">
+        <v>517393.2453</v>
+      </c>
+      <c r="J5">
+        <v>517409.0462</v>
+      </c>
+      <c r="K5">
+        <v>50</v>
+      </c>
+      <c r="L5">
+        <v>50</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>3</v>
+      </c>
+      <c r="O5">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>